<commit_message>
Updated catalog of LMU cars
</commit_message>
<xml_diff>
--- a/LmuCarAndTrackInfo.xlsx
+++ b/LmuCarAndTrackInfo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_src\sim-racing-sdk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204D3585-E536-41F7-8975-90367B0932AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DF6072-41EB-493F-8D01-8143D5D5EB77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7815" yWindow="2805" windowWidth="39915" windowHeight="16185" activeTab="1" xr2:uid="{13DF9C7F-C201-432D-A6DE-79F0069564C9}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{13DF9C7F-C201-432D-A6DE-79F0069564C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Cars" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="159">
   <si>
     <t>Class</t>
   </si>
@@ -478,6 +478,42 @@
   </si>
   <si>
     <t>School Circuit</t>
+  </si>
+  <si>
+    <t>Genesis</t>
+  </si>
+  <si>
+    <t>Genesis GMR-001</t>
+  </si>
+  <si>
+    <t>3.2L V8 Twin Turbo</t>
+  </si>
+  <si>
+    <t>LMP3</t>
+  </si>
+  <si>
+    <t>ADESS</t>
+  </si>
+  <si>
+    <t>ADESS-03</t>
+  </si>
+  <si>
+    <t>Duqueine 09</t>
+  </si>
+  <si>
+    <t>Duqueine</t>
+  </si>
+  <si>
+    <t>Ginetta</t>
+  </si>
+  <si>
+    <t>Ginetta G61-LT-P325-Evo</t>
+  </si>
+  <si>
+    <t>Ligier</t>
+  </si>
+  <si>
+    <t>Ligier JS P325</t>
   </si>
 </sst>
 </file>
@@ -856,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAF4C0E9-B717-44DD-9E2A-F8587A2DB755}">
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -954,7 +990,7 @@
         <v>17</v>
       </c>
       <c r="O2" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B2 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A2 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D2 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F2 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L2 &amp; ", LengthMm=" &amp; J2 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C2 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G2 &amp; ", PowerKw=" &amp; H2 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E2 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M2 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I2 &amp; ", WidthMm=" &amp; K2 &amp; "},"</f>
+        <f t="shared" ref="O2:O34" si="0">"new() { Category=" &amp; CHAR(34) &amp; B2 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A2 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D2 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F2 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L2 &amp; ", LengthMm=" &amp; J2 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C2 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G2 &amp; ", PowerKw=" &amp; H2 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E2 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M2 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I2 &amp; ", WidthMm=" &amp; K2 &amp; "},"</f>
         <v>new() { Category="LMDh", Class="HYP", DisplayName="Alpine A424", Engine="3.4L V6 Turbo", HeightMm=1055, LengthMm=5088, Manufacturer="Alpine", PowerBhp= 675, PowerKw=520, ResultCarType="Alpine A424", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=1992},</v>
       </c>
     </row>
@@ -999,7 +1035,7 @@
         <v>17</v>
       </c>
       <c r="O3" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B3 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A3 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D3 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F3 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L3 &amp; ", LengthMm=" &amp; J3 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C3 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G3 &amp; ", PowerKw=" &amp; H3 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E3 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M3 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I3 &amp; ", WidthMm=" &amp; K3 &amp; "},"</f>
+        <f t="shared" si="0"/>
         <v>new() { Category="LMH", Class="HYP", DisplayName="Aston Martin Valkyrie", Engine="6.5L Naturally Aspirated V12", HeightMm=1070, LengthMm=4500, Manufacturer="Aston Martin", PowerBhp= 670, PowerKw=500, ResultCarType="Aston Martin Valkyrie", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=1965},</v>
       </c>
     </row>
@@ -1044,7 +1080,7 @@
         <v>17</v>
       </c>
       <c r="O4" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B4 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A4 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D4 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F4 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L4 &amp; ", LengthMm=" &amp; J4 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C4 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G4 &amp; ", PowerKw=" &amp; H4 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E4 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M4 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I4 &amp; ", WidthMm=" &amp; K4 &amp; "},"</f>
+        <f t="shared" si="0"/>
         <v>new() { Category="LMDh", Class="HYP", DisplayName="BMW M Hybrid V8", Engine="4.0L V8 Twin Turbo", HeightMm=1200, LengthMm=4991, Manufacturer="BMW", PowerBhp= 650, PowerKw=485, ResultCarType="BMW M Hybrid V8", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=1994},</v>
       </c>
     </row>
@@ -1089,7 +1125,7 @@
         <v>17</v>
       </c>
       <c r="O5" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B5 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A5 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D5 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F5 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L5 &amp; ", LengthMm=" &amp; J5 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C5 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G5 &amp; ", PowerKw=" &amp; H5 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E5 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M5 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I5 &amp; ", WidthMm=" &amp; K5 &amp; "},"</f>
+        <f t="shared" si="0"/>
         <v>new() { Category="LMDh", Class="HYP", DisplayName="Cadillac V-Series.R", Engine="5.5L V8", HeightMm=1168, LengthMm=5100, Manufacturer="Cadillac", PowerBhp= 670, PowerKw=520, ResultCarType="Cadillac V-Series.R", Transmission="7 Speed Sequential", WeightKg=1046, WidthMm=2000},</v>
       </c>
     </row>
@@ -1134,7 +1170,7 @@
         <v>17</v>
       </c>
       <c r="O6" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B6 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A6 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D6 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F6 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L6 &amp; ", LengthMm=" &amp; J6 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C6 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G6 &amp; ", PowerKw=" &amp; H6 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E6 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M6 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I6 &amp; ", WidthMm=" &amp; K6 &amp; "},"</f>
+        <f t="shared" si="0"/>
         <v>new() { Category="LMH", Class="HYP", DisplayName="Ferrari 499P", Engine="3.0L V6 Twin Turbo", HeightMm=1055, LengthMm=5100, Manufacturer="Ferrari", PowerBhp= 670, PowerKw=500, ResultCarType="Ferrari 499P", Transmission="7 Speed Sequential", WeightKg=1057, WidthMm=2000},</v>
       </c>
     </row>
@@ -1143,44 +1179,44 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>149</v>
       </c>
       <c r="G7">
-        <v>670</v>
+        <v>690</v>
       </c>
       <c r="H7">
-        <v>520</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>1030</v>
       </c>
       <c r="J7">
-        <v>4991</v>
+        <v>5000</v>
       </c>
       <c r="K7">
         <v>2000</v>
       </c>
       <c r="L7">
-        <v>1224</v>
+        <v>1055</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
       </c>
       <c r="O7" t="str">
         <f>"new() { Category=" &amp; CHAR(34) &amp; B7 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A7 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D7 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F7 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L7 &amp; ", LengthMm=" &amp; J7 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C7 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G7 &amp; ", PowerKw=" &amp; H7 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E7 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M7 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I7 &amp; ", WidthMm=" &amp; K7 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Glickenhouse SCG 007", Engine="3.5L V8 Twin Turbo", HeightMm=1224, LengthMm=4991, Manufacturer="Glickenhaus", PowerBhp= 670, PowerKw=520, ResultCarType="Glickenhouse SCG 007", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <v>new() { Category="LMDh", Class="HYP", DisplayName="Genesis GMR-001", Engine="3.2L V8 Twin Turbo", HeightMm=1055, LengthMm=5000, Manufacturer="Genesis", PowerBhp= 690, PowerKw=0, ResultCarType="Genesis GMR-001", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1191,16 +1227,16 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G8">
         <v>670</v>
@@ -1212,20 +1248,20 @@
         <v>1030</v>
       </c>
       <c r="J8">
-        <v>5000</v>
+        <v>4991</v>
       </c>
       <c r="K8">
         <v>2000</v>
       </c>
       <c r="L8">
-        <v>1260</v>
+        <v>1224</v>
       </c>
       <c r="M8" t="s">
         <v>17</v>
       </c>
       <c r="O8" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B8 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A8 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D8 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F8 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L8 &amp; ", LengthMm=" &amp; J8 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C8 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G8 &amp; ", PowerKw=" &amp; H8 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E8 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M8 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I8 &amp; ", WidthMm=" &amp; K8 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Isotta Fraschini Tipo 6", Engine="3.0L V6 Turbo", HeightMm=1260, LengthMm=5000, Manufacturer="Isotta Fraschini", PowerBhp= 670, PowerKw=520, ResultCarType="Isotta Fraschini Tipo 6", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Glickenhouse SCG 007", Engine="3.5L V8 Twin Turbo", HeightMm=1224, LengthMm=4991, Manufacturer="Glickenhaus", PowerBhp= 670, PowerKw=520, ResultCarType="Glickenhouse SCG 007", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1233,19 +1269,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G9">
         <v>670</v>
@@ -1257,20 +1293,20 @@
         <v>1030</v>
       </c>
       <c r="J9">
-        <v>5100</v>
+        <v>5000</v>
       </c>
       <c r="K9">
         <v>2000</v>
       </c>
       <c r="L9">
-        <v>1170</v>
+        <v>1260</v>
       </c>
       <c r="M9" t="s">
         <v>17</v>
       </c>
       <c r="O9" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B9 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A9 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D9 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F9 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L9 &amp; ", LengthMm=" &amp; J9 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C9 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G9 &amp; ", PowerKw=" &amp; H9 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E9 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M9 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I9 &amp; ", WidthMm=" &amp; K9 &amp; "},"</f>
-        <v>new() { Category="LMDh", Class="HYP", DisplayName="Lamborghini SC63", Engine="3.8L V8 Twin Turbo", HeightMm=1170, LengthMm=5100, Manufacturer="Lamborghini", PowerBhp= 670, PowerKw=520, ResultCarType="Lamborghini SC63", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Isotta Fraschini Tipo 6", Engine="3.0L V6 Turbo", HeightMm=1260, LengthMm=5000, Manufacturer="Isotta Fraschini", PowerBhp= 670, PowerKw=520, ResultCarType="Isotta Fraschini Tipo 6", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1278,19 +1314,19 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G10">
         <v>670</v>
@@ -1302,20 +1338,20 @@
         <v>1030</v>
       </c>
       <c r="J10">
-        <v>4995</v>
+        <v>5100</v>
       </c>
       <c r="K10">
         <v>2000</v>
       </c>
       <c r="L10">
-        <v>1145</v>
+        <v>1170</v>
       </c>
       <c r="M10" t="s">
         <v>17</v>
       </c>
       <c r="O10" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B10 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A10 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D10 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F10 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L10 &amp; ", LengthMm=" &amp; J10 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C10 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G10 &amp; ", PowerKw=" &amp; H10 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E10 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M10 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I10 &amp; ", WidthMm=" &amp; K10 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Peugeot 9X8", Engine="2.6L V6 Twin Turbo", HeightMm=1145, LengthMm=4995, Manufacturer="Peugeot", PowerBhp= 670, PowerKw=520, ResultCarType="Peugeot 9X8", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMDh", Class="HYP", DisplayName="Lamborghini SC63", Engine="3.8L V8 Twin Turbo", HeightMm=1170, LengthMm=5100, Manufacturer="Lamborghini", PowerBhp= 670, PowerKw=520, ResultCarType="Lamborghini SC63", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1329,10 +1365,10 @@
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F11" t="s">
         <v>43</v>
@@ -1347,20 +1383,20 @@
         <v>1030</v>
       </c>
       <c r="J11">
-        <v>5000</v>
+        <v>4995</v>
       </c>
       <c r="K11">
-        <v>2080</v>
+        <v>2000</v>
       </c>
       <c r="L11">
-        <v>1180</v>
+        <v>1145</v>
       </c>
       <c r="M11" t="s">
         <v>17</v>
       </c>
       <c r="O11" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B11 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A11 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D11 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F11 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L11 &amp; ", LengthMm=" &amp; J11 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C11 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G11 &amp; ", PowerKw=" &amp; H11 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E11 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M11 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I11 &amp; ", WidthMm=" &amp; K11 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Peugeot 9X8 2024", Engine="2.6L V6 Twin Turbo", HeightMm=1180, LengthMm=5000, Manufacturer="Peugeot", PowerBhp= 670, PowerKw=520, ResultCarType="Peugeot 9X8 2024", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2080},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Peugeot 9X8", Engine="2.6L V6 Twin Turbo", HeightMm=1145, LengthMm=4995, Manufacturer="Peugeot", PowerBhp= 670, PowerKw=520, ResultCarType="Peugeot 9X8", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -1371,41 +1407,41 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G12">
         <v>670</v>
       </c>
       <c r="H12">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="I12">
         <v>1030</v>
       </c>
       <c r="J12">
-        <v>5100</v>
+        <v>5000</v>
       </c>
       <c r="K12">
-        <v>2000</v>
+        <v>2080</v>
       </c>
       <c r="L12">
-        <v>1060</v>
+        <v>1180</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="O12" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B12 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A12 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D12 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F12 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L12 &amp; ", LengthMm=" &amp; J12 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C12 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G12 &amp; ", PowerKw=" &amp; H12 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E12 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M12 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I12 &amp; ", WidthMm=" &amp; K12 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Porsche 963", Engine="4.6L V8 Twin Turbo", HeightMm=1060, LengthMm=5100, Manufacturer="Porsche", PowerBhp= 670, PowerKw=500, ResultCarType="Porsche 963", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Peugeot 9X8 2024", Engine="2.6L V6 Twin Turbo", HeightMm=1180, LengthMm=5000, Manufacturer="Peugeot", PowerBhp= 670, PowerKw=520, ResultCarType="Peugeot 9X8 2024", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2080},</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1416,16 +1452,16 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G13">
         <v>670</v>
@@ -1434,23 +1470,23 @@
         <v>500</v>
       </c>
       <c r="I13">
-        <v>1062</v>
+        <v>1030</v>
       </c>
       <c r="J13">
-        <v>4900</v>
+        <v>5100</v>
       </c>
       <c r="K13">
         <v>2000</v>
       </c>
       <c r="L13">
-        <v>1150</v>
+        <v>1060</v>
       </c>
       <c r="M13" t="s">
         <v>17</v>
       </c>
       <c r="O13" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B13 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A13 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D13 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F13 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L13 &amp; ", LengthMm=" &amp; J13 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C13 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G13 &amp; ", PowerKw=" &amp; H13 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E13 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M13 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I13 &amp; ", WidthMm=" &amp; K13 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Toyota GR010-Hybrid", Engine="3.5L V6 Twin Turbo", HeightMm=1150, LengthMm=4900, Manufacturer="Toyota", PowerBhp= 670, PowerKw=500, ResultCarType="Toyota GR010-Hybrid", Transmission="7 Speed Sequential", WeightKg=1062, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Porsche 963", Engine="4.6L V8 Twin Turbo", HeightMm=1060, LengthMm=5100, Manufacturer="Porsche", PowerBhp= 670, PowerKw=500, ResultCarType="Porsche 963", Transmission="7 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1461,86 +1497,86 @@
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G14">
         <v>670</v>
       </c>
       <c r="H14">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="I14">
-        <v>1030</v>
+        <v>1062</v>
       </c>
       <c r="J14">
-        <v>5000</v>
+        <v>4900</v>
       </c>
       <c r="K14">
         <v>2000</v>
       </c>
       <c r="L14">
-        <v>1168</v>
+        <v>1150</v>
       </c>
       <c r="M14" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="O14" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B14 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A14 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D14 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F14 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L14 &amp; ", LengthMm=" &amp; J14 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C14 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G14 &amp; ", PowerKw=" &amp; H14 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E14 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M14 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I14 &amp; ", WidthMm=" &amp; K14 &amp; "},"</f>
-        <v>new() { Category="LMH", Class="HYP", DisplayName="Vanwall Vandervell 680", Engine="4.5L V8", HeightMm=1168, LengthMm=5000, Manufacturer="Vanwall", PowerBhp= 670, PowerKw=520, ResultCarType="Vanwall Vandervell 680", Transmission="6 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Toyota GR010-Hybrid", Engine="3.5L V6 Twin Turbo", HeightMm=1150, LengthMm=4900, Manufacturer="Toyota", PowerBhp= 670, PowerKw=500, ResultCarType="Toyota GR010-Hybrid", Transmission="7 Speed Sequential", WeightKg=1062, WidthMm=2000},</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G15">
-        <v>603</v>
+        <v>670</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="I15">
-        <v>930</v>
+        <v>1030</v>
       </c>
       <c r="J15">
-        <v>4745</v>
+        <v>5000</v>
       </c>
       <c r="K15">
-        <v>1895</v>
+        <v>2000</v>
       </c>
       <c r="L15">
-        <v>1045</v>
+        <v>1168</v>
       </c>
       <c r="M15" t="s">
         <v>54</v>
       </c>
       <c r="O15" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B15 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A15 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D15 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F15 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L15 &amp; ", LengthMm=" &amp; J15 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C15 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G15 &amp; ", PowerKw=" &amp; H15 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E15 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M15 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I15 &amp; ", WidthMm=" &amp; K15 &amp; "},"</f>
-        <v>new() { Category="LMP2", Class="LMP2", DisplayName="ORECA 07 Gibson 2023", Engine="4.2l V8", HeightMm=1045, LengthMm=4745, Manufacturer="ORECA", PowerBhp= 603, PowerKw=0, ResultCarType="ORECA 07 Gibson 2023", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1895},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMH", Class="HYP", DisplayName="Vanwall Vandervell 680", Engine="4.5L V8", HeightMm=1168, LengthMm=5000, Manufacturer="Vanwall", PowerBhp= 670, PowerKw=520, ResultCarType="Vanwall Vandervell 680", Transmission="6 Speed Sequential", WeightKg=1030, WidthMm=2000},</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1554,10 +1590,10 @@
         <v>56</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F16" t="s">
         <v>57</v>
@@ -1584,413 +1620,413 @@
         <v>54</v>
       </c>
       <c r="O16" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B16 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A16 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D16 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F16 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L16 &amp; ", LengthMm=" &amp; J16 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C16 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G16 &amp; ", PowerKw=" &amp; H16 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E16 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M16 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I16 &amp; ", WidthMm=" &amp; K16 &amp; "},"</f>
-        <v>new() { Category="LMP2", Class="LMP2", DisplayName="ORECA 07 Gibson 2024", Engine="4.2l V8", HeightMm=1045, LengthMm=4745, Manufacturer="ORECA", PowerBhp= 603, PowerKw=0, ResultCarType="ORECA 07 Gibson 2024", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1895},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP2", Class="LMP2", DisplayName="ORECA 07 Gibson 2023", Engine="4.2l V8", HeightMm=1045, LengthMm=4745, Manufacturer="ORECA", PowerBhp= 603, PowerKw=0, ResultCarType="ORECA 07 Gibson 2023", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1895},</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G17">
-        <v>500</v>
+        <v>603</v>
       </c>
       <c r="H17">
         <v>0</v>
       </c>
       <c r="I17">
-        <v>1245</v>
+        <v>930</v>
       </c>
       <c r="J17">
-        <v>4665</v>
+        <v>4745</v>
       </c>
       <c r="K17">
-        <v>2153</v>
+        <v>1895</v>
       </c>
       <c r="L17">
-        <v>1274</v>
+        <v>1045</v>
       </c>
       <c r="M17" t="s">
         <v>54</v>
       </c>
       <c r="O17" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B17 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A17 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D17 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F17 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L17 &amp; ", LengthMm=" &amp; J17 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C17 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G17 &amp; ", PowerKw=" &amp; H17 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E17 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M17 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I17 &amp; ", WidthMm=" &amp; K17 &amp; "},"</f>
-        <v>new() { Category="GTE", Class="GTE", DisplayName="Aston Martin Vantage AMR", Engine="4.0L V8 Turbo", HeightMm=1274, LengthMm=4665, Manufacturer="Aston Martin", PowerBhp= 500, PowerKw=0, ResultCarType="Aston Martin Vantage AMR", Transmission="6 Speed Sequential", WeightKg=1245, WidthMm=2153},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP2", Class="LMP2", DisplayName="ORECA 07 Gibson 2024", Engine="4.2l V8", HeightMm=1045, LengthMm=4745, Manufacturer="ORECA", PowerBhp= 603, PowerKw=0, ResultCarType="ORECA 07 Gibson 2024", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1895},</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>152</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>152</v>
       </c>
       <c r="F18" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="G18">
-        <v>500</v>
+        <v>470</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1245</v>
+        <v>930</v>
       </c>
       <c r="J18">
-        <v>4614</v>
+        <v>4643</v>
       </c>
       <c r="K18">
-        <v>2050</v>
+        <v>1890</v>
       </c>
       <c r="L18">
-        <v>1090</v>
+        <v>1050</v>
       </c>
       <c r="M18" t="s">
         <v>54</v>
       </c>
       <c r="O18" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B18 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A18 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D18 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F18 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L18 &amp; ", LengthMm=" &amp; J18 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C18 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G18 &amp; ", PowerKw=" &amp; H18 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E18 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M18 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I18 &amp; ", WidthMm=" &amp; K18 &amp; "},"</f>
-        <v>new() { Category="GTE", Class="GTE", DisplayName="Ferrari 488 GTE Evo", Engine="4.0L V8 Turbo", HeightMm=1090, LengthMm=4614, Manufacturer="Ferrari", PowerBhp= 500, PowerKw=0, ResultCarType="Ferrari 488 GTE Evo", Transmission="6 Speed Sequential", WeightKg=1245, WidthMm=2050},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP3", Class="LMP3", DisplayName="ADESS-03", Engine="3.5L V6 Twin Turbo", HeightMm=1050, LengthMm=4643, Manufacturer="ADESS", PowerBhp= 470, PowerKw=0, ResultCarType="ADESS-03", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1890},</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>154</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="E19" t="s">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="F19" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G19">
-        <v>510</v>
+        <v>470</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>1243</v>
+        <v>930</v>
       </c>
       <c r="J19">
-        <v>4557</v>
+        <v>4643</v>
       </c>
       <c r="K19">
-        <v>2042</v>
+        <v>1890</v>
       </c>
       <c r="L19">
-        <v>1250</v>
+        <v>1050</v>
       </c>
       <c r="M19" t="s">
         <v>54</v>
       </c>
       <c r="O19" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B19 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A19 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D19 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F19 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L19 &amp; ", LengthMm=" &amp; J19 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C19 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G19 &amp; ", PowerKw=" &amp; H19 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E19 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M19 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I19 &amp; ", WidthMm=" &amp; K19 &amp; "},"</f>
-        <v>new() { Category="GTE", Class="GTE", DisplayName="Porsche 911 RSR-I9", Engine="4.0L Flat Six", HeightMm=1250, LengthMm=4557, Manufacturer="Porsche", PowerBhp= 510, PowerKw=0, ResultCarType="Porsche 911 RSR-I9", Transmission="6 Speed Sequential", WeightKg=1243, WidthMm=2042},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP3", Class="LMP3", DisplayName="Duqueine 09", Engine="3.5L V6 Twin Turbo", HeightMm=1050, LengthMm=4643, Manufacturer="Duqueine", PowerBhp= 470, PowerKw=0, ResultCarType="Duqueine 09", Transmission="6 Speed Sequential", WeightKg=930, WidthMm=1890},</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="D20" t="s">
-        <v>67</v>
+        <v>156</v>
       </c>
       <c r="E20" t="s">
-        <v>67</v>
+        <v>156</v>
       </c>
       <c r="F20" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="G20">
-        <v>500</v>
+        <v>470</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>1240</v>
+        <v>950</v>
       </c>
       <c r="J20">
-        <v>4630</v>
+        <v>4605</v>
       </c>
       <c r="K20">
-        <v>2053</v>
+        <v>1900</v>
       </c>
       <c r="L20">
-        <v>1148</v>
+        <v>1050</v>
       </c>
       <c r="M20" t="s">
         <v>54</v>
       </c>
       <c r="O20" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B20 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A20 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D20 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F20 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L20 &amp; ", LengthMm=" &amp; J20 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C20 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G20 &amp; ", PowerKw=" &amp; H20 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E20 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M20 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I20 &amp; ", WidthMm=" &amp; K20 &amp; "},"</f>
-        <v>new() { Category="GTE", Class="GTE", DisplayName="Chevrolet Corvette C8.R", Engine="5.0L V8", HeightMm=1148, LengthMm=4630, Manufacturer="Chevrolet", PowerBhp= 500, PowerKw=0, ResultCarType="Chevrolet Corvette C8.R", Transmission="6 Speed Sequential", WeightKg=1240, WidthMm=2053},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP3", Class="LMP3", DisplayName="Ginetta G61-LT-P325-Evo", Engine="3.5L V6 Twin Turbo", HeightMm=1050, LengthMm=4605, Manufacturer="Ginetta", PowerBhp= 470, PowerKw=0, ResultCarType="Ginetta G61-LT-P325-Evo", Transmission="6 Speed Sequential", WeightKg=950, WidthMm=1900},</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>150</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>158</v>
       </c>
       <c r="E21" t="s">
-        <v>71</v>
+        <v>158</v>
       </c>
       <c r="F21" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="G21">
-        <v>535</v>
+        <v>470</v>
       </c>
       <c r="H21">
         <v>0</v>
       </c>
       <c r="I21">
-        <v>1306</v>
+        <v>950</v>
       </c>
       <c r="J21">
-        <v>4616</v>
+        <v>4605</v>
       </c>
       <c r="K21">
-        <v>2049</v>
+        <v>1900</v>
       </c>
       <c r="L21">
-        <v>1144</v>
+        <v>1180</v>
       </c>
       <c r="M21" t="s">
         <v>54</v>
       </c>
       <c r="O21" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B21 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A21 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D21 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F21 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L21 &amp; ", LengthMm=" &amp; J21 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C21 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G21 &amp; ", PowerKw=" &amp; H21 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E21 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M21 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I21 &amp; ", WidthMm=" &amp; K21 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Aston Martin Vantage AMR LMGT3", Engine="4.0L V8 Twin Turbo", HeightMm=1144, LengthMm=4616, Manufacturer="Aston Martin", PowerBhp= 535, PowerKw=0, ResultCarType="Aston Martin Vantage AMR LMGT3", Transmission="6 Speed Sequential", WeightKg=1306, WidthMm=2049},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMP3", Class="LMP3", DisplayName="Ligier JS P325", Engine="3.5L V6 Twin Turbo", HeightMm=1180, LengthMm=4605, Manufacturer="Ligier", PowerBhp= 470, PowerKw=0, ResultCarType="Ligier JS P325", Transmission="6 Speed Sequential", WeightKg=950, WidthMm=1900},</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E22" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="F22" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="G22">
-        <v>590</v>
+        <v>500</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>1339</v>
+        <v>1245</v>
       </c>
       <c r="J22">
-        <v>5020</v>
+        <v>4665</v>
       </c>
       <c r="K22">
-        <v>2040</v>
+        <v>2153</v>
       </c>
       <c r="L22">
-        <v>1308</v>
+        <v>1274</v>
       </c>
       <c r="M22" t="s">
         <v>54</v>
       </c>
       <c r="O22" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B22 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A22 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D22 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F22 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L22 &amp; ", LengthMm=" &amp; J22 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C22 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G22 &amp; ", PowerKw=" &amp; H22 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E22 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M22 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I22 &amp; ", WidthMm=" &amp; K22 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="BMW M4 LMGT3", Engine="3.0L Straight Six Turbo", HeightMm=1308, LengthMm=5020, Manufacturer="BMW", PowerBhp= 590, PowerKw=0, ResultCarType="BMW M4 LMGT3", Transmission="6 Speed Sequential", WeightKg=1339, WidthMm=2040},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="GTE", Class="GTE", DisplayName="Aston Martin Vantage AMR", Engine="4.0L V8 Turbo", HeightMm=1274, LengthMm=4665, Manufacturer="Aston Martin", PowerBhp= 500, PowerKw=0, ResultCarType="Aston Martin Vantage AMR", Transmission="6 Speed Sequential", WeightKg=1245, WidthMm=2153},</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="E23" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F23" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="G23">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>1344</v>
+        <v>1245</v>
       </c>
       <c r="J23">
-        <v>4630</v>
+        <v>4614</v>
       </c>
       <c r="K23">
         <v>2050</v>
       </c>
       <c r="L23">
-        <v>1148</v>
+        <v>1090</v>
       </c>
       <c r="M23" t="s">
         <v>54</v>
       </c>
       <c r="O23" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B23 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A23 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D23 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F23 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L23 &amp; ", LengthMm=" &amp; J23 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C23 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G23 &amp; ", PowerKw=" &amp; H23 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E23 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M23 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I23 &amp; ", WidthMm=" &amp; K23 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Corevette Z06 LMGT3.R", Engine="5.5L V8", HeightMm=1148, LengthMm=4630, Manufacturer="Corvette", PowerBhp= 600, PowerKw=0, ResultCarType="Corevette Z06 LMGT3.R", Transmission="6 Speed Sequential", WeightKg=1344, WidthMm=2050},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="GTE", Class="GTE", DisplayName="Ferrari 488 GTE Evo", Engine="4.0L V8 Turbo", HeightMm=1090, LengthMm=4614, Manufacturer="Ferrari", PowerBhp= 500, PowerKw=0, ResultCarType="Ferrari 488 GTE Evo", Transmission="6 Speed Sequential", WeightKg=1245, WidthMm=2050},</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="E24" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F24" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="G24">
-        <v>600</v>
+        <v>510</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>1341</v>
+        <v>1243</v>
       </c>
       <c r="J24">
-        <v>4565</v>
+        <v>4557</v>
       </c>
       <c r="K24">
-        <v>2050</v>
+        <v>2042</v>
       </c>
       <c r="L24">
-        <v>1191</v>
+        <v>1250</v>
       </c>
       <c r="M24" t="s">
         <v>54</v>
       </c>
       <c r="O24" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B24 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A24 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D24 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F24 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L24 &amp; ", LengthMm=" &amp; J24 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C24 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G24 &amp; ", PowerKw=" &amp; H24 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E24 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M24 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I24 &amp; ", WidthMm=" &amp; K24 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Ferrari 296 LMGT3", Engine="2.9L V6 Turbo", HeightMm=1191, LengthMm=4565, Manufacturer="Ferrari", PowerBhp= 600, PowerKw=0, ResultCarType="Ferrari 296 LMGT3", Transmission="6 Speed Sequential", WeightKg=1341, WidthMm=2050},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="GTE", Class="GTE", DisplayName="Porsche 911 RSR-I9", Engine="4.0L Flat Six", HeightMm=1250, LengthMm=4557, Manufacturer="Porsche", PowerBhp= 510, PowerKw=0, ResultCarType="Porsche 911 RSR-I9", Transmission="6 Speed Sequential", WeightKg=1243, WidthMm=2042},</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="E25" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F25" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G25">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25">
-        <v>1329</v>
+        <v>1240</v>
       </c>
       <c r="J25">
-        <v>4797</v>
+        <v>4630</v>
       </c>
       <c r="K25">
-        <v>1918</v>
+        <v>2053</v>
       </c>
       <c r="L25">
-        <v>1392</v>
+        <v>1148</v>
       </c>
       <c r="M25" t="s">
         <v>54</v>
       </c>
       <c r="O25" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B25 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A25 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D25 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F25 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L25 &amp; ", LengthMm=" &amp; J25 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C25 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G25 &amp; ", PowerKw=" &amp; H25 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E25 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M25 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I25 &amp; ", WidthMm=" &amp; K25 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Ford Mustang LMGT3", Engine="5.4L V8", HeightMm=1392, LengthMm=4797, Manufacturer="Ford", PowerBhp= 550, PowerKw=0, ResultCarType="Ford Mustang LMGT3", Transmission="6 Speed Sequential", WeightKg=1329, WidthMm=1918},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="GTE", Class="GTE", DisplayName="Chevrolet Corvette C8.R", Engine="5.0L V8", HeightMm=1148, LengthMm=4630, Manufacturer="Chevrolet", PowerBhp= 500, PowerKw=0, ResultCarType="Chevrolet Corvette C8.R", Transmission="6 Speed Sequential", WeightKg=1240, WidthMm=2053},</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -2001,41 +2037,41 @@
         <v>70</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E26" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F26" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="G26">
-        <v>640</v>
+        <v>535</v>
       </c>
       <c r="H26">
         <v>0</v>
       </c>
       <c r="I26">
-        <v>1355</v>
+        <v>1306</v>
       </c>
       <c r="J26">
-        <v>4551</v>
+        <v>4616</v>
       </c>
       <c r="K26">
-        <v>2221</v>
+        <v>2049</v>
       </c>
       <c r="L26">
-        <v>1165</v>
+        <v>1144</v>
       </c>
       <c r="M26" t="s">
         <v>54</v>
       </c>
       <c r="O26" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B26 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A26 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D26 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F26 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L26 &amp; ", LengthMm=" &amp; J26 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C26 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G26 &amp; ", PowerKw=" &amp; H26 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E26 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M26 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I26 &amp; ", WidthMm=" &amp; K26 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Lamborghini Huracan LMGT3 Evo2", Engine="V10 Naturally Aspirated", HeightMm=1165, LengthMm=4551, Manufacturer="Lamborghini", PowerBhp= 640, PowerKw=0, ResultCarType="Lamborghini Huracan LMGT3 Evo2", Transmission="6 Speed Sequential", WeightKg=1355, WidthMm=2221},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Aston Martin Vantage AMR LMGT3", Engine="4.0L V8 Twin Turbo", HeightMm=1144, LengthMm=4616, Manufacturer="Aston Martin", PowerBhp= 535, PowerKw=0, ResultCarType="Aston Martin Vantage AMR LMGT3", Transmission="6 Speed Sequential", WeightKg=1306, WidthMm=2049},</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -2046,41 +2082,41 @@
         <v>70</v>
       </c>
       <c r="C27" t="s">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E27" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="F27" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G27">
-        <v>500</v>
+        <v>590</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27">
-        <v>1355</v>
+        <v>1339</v>
       </c>
       <c r="J27">
-        <v>4846</v>
+        <v>5020</v>
       </c>
       <c r="K27">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="L27">
-        <v>1271</v>
+        <v>1308</v>
       </c>
       <c r="M27" t="s">
         <v>54</v>
       </c>
       <c r="O27" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B27 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A27 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D27 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F27 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L27 &amp; ", LengthMm=" &amp; J27 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C27 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G27 &amp; ", PowerKw=" &amp; H27 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E27 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M27 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I27 &amp; ", WidthMm=" &amp; K27 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Lexus RC F LMGT3", Engine="5.4L V8", HeightMm=1271, LengthMm=4846, Manufacturer="Lexus", PowerBhp= 500, PowerKw=0, ResultCarType="Lexus RCF LMGT3", Transmission="6 Speed Sequential", WeightKg=1355, WidthMm=2030},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="BMW M4 LMGT3", Engine="3.0L Straight Six Turbo", HeightMm=1308, LengthMm=5020, Manufacturer="BMW", PowerBhp= 590, PowerKw=0, ResultCarType="BMW M4 LMGT3", Transmission="6 Speed Sequential", WeightKg=1339, WidthMm=2040},</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -2091,16 +2127,16 @@
         <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D28" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E28" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="G28">
         <v>600</v>
@@ -2109,23 +2145,23 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="J28">
-        <v>4543</v>
+        <v>4630</v>
       </c>
       <c r="K28">
-        <v>2161</v>
+        <v>2050</v>
       </c>
       <c r="L28">
-        <v>1196</v>
+        <v>1148</v>
       </c>
       <c r="M28" t="s">
         <v>54</v>
       </c>
       <c r="O28" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B28 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A28 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D28 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F28 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L28 &amp; ", LengthMm=" &amp; J28 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C28 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G28 &amp; ", PowerKw=" &amp; H28 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E28 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M28 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I28 &amp; ", WidthMm=" &amp; K28 &amp; "},"</f>
-        <v>new() { Category="LMGT3", Class="GT3", DisplayName="McLaren 720S LMGT3 Evo", Engine="4.0L V8 Twin Turbo", HeightMm=1196, LengthMm=4543, Manufacturer="McLaren", PowerBhp= 600, PowerKw=0, ResultCarType="McLaren 720S LMGT3 Evo", Transmission="6 Speed Sequential", WeightKg=1345, WidthMm=2161},</v>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Corevette Z06 LMGT3.R", Engine="5.5L V8", HeightMm=1148, LengthMm=4630, Manufacturer="Corvette", PowerBhp= 600, PowerKw=0, ResultCarType="Corevette Z06 LMGT3.R", Transmission="6 Speed Sequential", WeightKg=1344, WidthMm=2050},</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -2136,40 +2172,265 @@
         <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E29" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="F29" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="G29">
-        <v>565</v>
+        <v>600</v>
       </c>
       <c r="H29">
         <v>0</v>
       </c>
       <c r="I29">
-        <v>1317</v>
+        <v>1341</v>
       </c>
       <c r="J29">
-        <v>4619</v>
+        <v>4565</v>
       </c>
       <c r="K29">
         <v>2050</v>
       </c>
       <c r="L29">
-        <v>1279</v>
+        <v>1191</v>
       </c>
       <c r="M29" t="s">
         <v>54</v>
       </c>
       <c r="O29" t="str">
-        <f>"new() { Category=" &amp; CHAR(34) &amp; B29 &amp; CHAR(34) &amp; ", Class=" &amp; CHAR(34) &amp; A29 &amp; CHAR(34) &amp; ", DisplayName=" &amp; CHAR(34) &amp; D29 &amp; CHAR(34) &amp; ", Engine=" &amp; CHAR(34) &amp; F29 &amp; CHAR(34) &amp; ", HeightMm=" &amp; L29 &amp; ", LengthMm=" &amp; J29 &amp; ", Manufacturer=" &amp; CHAR(34) &amp; C29 &amp; CHAR(34) &amp; ", PowerBhp= " &amp; G29 &amp; ", PowerKw=" &amp; H29 &amp; ", ResultCarType=" &amp; CHAR(34) &amp; E29 &amp; CHAR(34) &amp; ", Transmission=" &amp; CHAR(34) &amp; M29 &amp; CHAR(34) &amp; ", WeightKg=" &amp; I29 &amp; ", WidthMm=" &amp; K29 &amp; "},"</f>
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Ferrari 296 LMGT3", Engine="2.9L V6 Turbo", HeightMm=1191, LengthMm=4565, Manufacturer="Ferrari", PowerBhp= 600, PowerKw=0, ResultCarType="Ferrari 296 LMGT3", Transmission="6 Speed Sequential", WeightKg=1341, WidthMm=2050},</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" t="s">
+        <v>80</v>
+      </c>
+      <c r="G30">
+        <v>550</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>1329</v>
+      </c>
+      <c r="J30">
+        <v>4797</v>
+      </c>
+      <c r="K30">
+        <v>1918</v>
+      </c>
+      <c r="L30">
+        <v>1392</v>
+      </c>
+      <c r="M30" t="s">
+        <v>54</v>
+      </c>
+      <c r="O30" t="str">
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Ford Mustang LMGT3", Engine="5.4L V8", HeightMm=1392, LengthMm=4797, Manufacturer="Ford", PowerBhp= 550, PowerKw=0, ResultCarType="Ford Mustang LMGT3", Transmission="6 Speed Sequential", WeightKg=1329, WidthMm=1918},</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" t="s">
+        <v>81</v>
+      </c>
+      <c r="F31" t="s">
+        <v>82</v>
+      </c>
+      <c r="G31">
+        <v>640</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>1355</v>
+      </c>
+      <c r="J31">
+        <v>4551</v>
+      </c>
+      <c r="K31">
+        <v>2221</v>
+      </c>
+      <c r="L31">
+        <v>1165</v>
+      </c>
+      <c r="M31" t="s">
+        <v>54</v>
+      </c>
+      <c r="O31" t="str">
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Lamborghini Huracan LMGT3 Evo2", Engine="V10 Naturally Aspirated", HeightMm=1165, LengthMm=4551, Manufacturer="Lamborghini", PowerBhp= 640, PowerKw=0, ResultCarType="Lamborghini Huracan LMGT3 Evo2", Transmission="6 Speed Sequential", WeightKg=1355, WidthMm=2221},</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" t="s">
+        <v>84</v>
+      </c>
+      <c r="E32" t="s">
+        <v>85</v>
+      </c>
+      <c r="F32" t="s">
+        <v>80</v>
+      </c>
+      <c r="G32">
+        <v>500</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>1355</v>
+      </c>
+      <c r="J32">
+        <v>4846</v>
+      </c>
+      <c r="K32">
+        <v>2030</v>
+      </c>
+      <c r="L32">
+        <v>1271</v>
+      </c>
+      <c r="M32" t="s">
+        <v>54</v>
+      </c>
+      <c r="O32" t="str">
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="Lexus RC F LMGT3", Engine="5.4L V8", HeightMm=1271, LengthMm=4846, Manufacturer="Lexus", PowerBhp= 500, PowerKw=0, ResultCarType="Lexus RCF LMGT3", Transmission="6 Speed Sequential", WeightKg=1355, WidthMm=2030},</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" t="s">
+        <v>87</v>
+      </c>
+      <c r="E33" t="s">
+        <v>87</v>
+      </c>
+      <c r="F33" t="s">
+        <v>40</v>
+      </c>
+      <c r="G33">
+        <v>600</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>1345</v>
+      </c>
+      <c r="J33">
+        <v>4543</v>
+      </c>
+      <c r="K33">
+        <v>2161</v>
+      </c>
+      <c r="L33">
+        <v>1196</v>
+      </c>
+      <c r="M33" t="s">
+        <v>54</v>
+      </c>
+      <c r="O33" t="str">
+        <f t="shared" si="0"/>
+        <v>new() { Category="LMGT3", Class="GT3", DisplayName="McLaren 720S LMGT3 Evo", Engine="4.0L V8 Twin Turbo", HeightMm=1196, LengthMm=4543, Manufacturer="McLaren", PowerBhp= 600, PowerKw=0, ResultCarType="McLaren 720S LMGT3 Evo", Transmission="6 Speed Sequential", WeightKg=1345, WidthMm=2161},</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>69</v>
+      </c>
+      <c r="B34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" t="s">
+        <v>88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>88</v>
+      </c>
+      <c r="F34" t="s">
+        <v>89</v>
+      </c>
+      <c r="G34">
+        <v>565</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>1317</v>
+      </c>
+      <c r="J34">
+        <v>4619</v>
+      </c>
+      <c r="K34">
+        <v>2050</v>
+      </c>
+      <c r="L34">
+        <v>1279</v>
+      </c>
+      <c r="M34" t="s">
+        <v>54</v>
+      </c>
+      <c r="O34" t="str">
+        <f t="shared" si="0"/>
         <v>new() { Category="LMGT3", Class="GT3", DisplayName="Porsche 911 GT3 R LMGT3", Engine="4.2L Straight Six", HeightMm=1279, LengthMm=4619, Manufacturer="Porsche", PowerBhp= 565, PowerKw=0, ResultCarType="Porsche 911 GT3 R LMGT3", Transmission="6 Speed Sequential", WeightKg=1317, WidthMm=2050},</v>
       </c>
     </row>

</xml_diff>